<commit_message>
[auto-snapshot] 2026-04-15 00:00 | onda-hompage | 416 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강남_PT.xlsx
+++ b/naver-place-crawler/results_health/강남_PT.xlsx
@@ -417,16 +417,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
@@ -559,34 +559,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>청담짐 PT</t>
+          <t>헬스보이짐 필라걸 학동역점</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>cheongdamgym8@naver.com</t>
+          <t>healthboygym37@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1332-0757</t>
+          <t>0507-1446-9059</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 도산대로81길 8 지하1층</t>
+          <t>서울특별시 강남구 학동로 171 삼익악기빌딩 B1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/cheongdamgym8</t>
+          <t>https://blog.naver.com/healthboygym37</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -612,7 +612,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>70</v>
+        <v>2330</v>
       </c>
       <c r="Q2" t="n">
-        <v>89</v>
+        <v>1057</v>
       </c>
       <c r="R2" t="n">
-        <v>159</v>
+        <v>3387</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -636,12 +636,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1729496529</t>
+          <t>1739218540</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1729496529</t>
+          <t>https://m.place.naver.com/place/1739218540</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -653,39 +653,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>웰앤피트니스 강남점</t>
+          <t>엑스퍼티짐 헬스 골프 역삼점</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>wellandfitness_gn@naver.com</t>
+          <t>expurty@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1462-7594</t>
+          <t>0507-1338-8250</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 언주로 563 원에디션 강남 B1층 B127호</t>
+          <t>서울특별시 강남구 테헤란로25길 7 창성재단빌딩 B1층 헬스 B2층 골프</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://wellandfitnessgn.co.kr/</t>
+          <t>https://blog.naver.com/expurty</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -706,7 +706,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>473</v>
+        <v>574</v>
       </c>
       <c r="Q3" t="n">
-        <v>269</v>
+        <v>590</v>
       </c>
       <c r="R3" t="n">
-        <v>742</v>
+        <v>1164</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,12 +730,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1596087105</t>
+          <t>1327900562</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1596087105</t>
+          <t>https://m.place.naver.com/place/1327900562</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -747,39 +747,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>헬스장</t>
+          <t>스포츠시설</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>팀버핏 도곡</t>
+          <t>에이블짐 강남역점</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>jhjh5508@naver.com</t>
+          <t>ablegym39@naver.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1352-1412</t>
+          <t>0507-1352-2640</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 언주로30길 21 B2층 B201-2호</t>
+          <t>서울특별시 강남구 강남대로 382 B2 에이블짐 강남역점</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.teambutfit.com/</t>
+          <t>https://blog.naver.com/ablegym39</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -809,13 +809,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>302</v>
+        <v>4576</v>
       </c>
       <c r="Q4" t="n">
-        <v>80</v>
+        <v>3295</v>
       </c>
       <c r="R4" t="n">
-        <v>382</v>
+        <v>7871</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -824,12 +824,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1114610716</t>
+          <t>1958479504</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1114610716</t>
+          <t>https://m.place.naver.com/place/1958479504</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -846,29 +846,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>에이블짐 강남역점</t>
+          <t>헬스보이짐 강남역점</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ablegym39@naver.com</t>
+          <t>healthboy352@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0507-1352-2640</t>
+          <t>0507-1443-0244</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 강남대로 382 B2 에이블짐 강남역점</t>
+          <t>서울특별시 강남구 테헤란로2길 27 패스트파이브빌딩 지하1층~지하2층</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ablegym39</t>
+          <t>https://blog.naver.com/healthboy352/224048963164</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -903,13 +903,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>4574</v>
+        <v>1117</v>
       </c>
       <c r="Q5" t="n">
-        <v>3287</v>
+        <v>1517</v>
       </c>
       <c r="R5" t="n">
-        <v>7861</v>
+        <v>2634</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -918,12 +918,12 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1958479504</t>
+          <t>1650445992</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1958479504</t>
+          <t>https://m.place.naver.com/place/1650445992</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -940,29 +940,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>헬스보이짐 강남역점</t>
+          <t>밸류온피트니스 헬스&amp;PT 역삼점</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>healthboy352@naver.com</t>
+          <t>pingpingwa@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0507-1443-0244</t>
+          <t>0507-1417-1245</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 테헤란로2길 27 패스트파이브빌딩 지하1층~지하2층</t>
+          <t>서울특별시 강남구 언주로 329 지하1층</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboy352/224048963164</t>
+          <t>https://blog.naver.com/pingpingwa</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -997,13 +997,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>1116</v>
+        <v>375</v>
       </c>
       <c r="Q6" t="n">
-        <v>1515</v>
+        <v>1527</v>
       </c>
       <c r="R6" t="n">
-        <v>2631</v>
+        <v>1902</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1012,12 +1012,12 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1650445992</t>
+          <t>1116991775</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1650445992</t>
+          <t>https://m.place.naver.com/place/1116991775</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1029,34 +1029,34 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>밸류온피트니스 헬스&amp;PT 역삼점</t>
+          <t>바디쉬휘트니스 언주역점</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pingpingwa@naver.com</t>
+          <t>bodyshe_1@naver.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0507-1417-1245</t>
+          <t>0507-1417-1995</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 언주로 329 지하1층</t>
+          <t>서울특별시 강남구 논현로 611 지하1층</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/pingpingwa</t>
+          <t>https://blog.naver.com/bodyshe_1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1091,13 +1091,13 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>375</v>
+        <v>1030</v>
       </c>
       <c r="Q7" t="n">
-        <v>1536</v>
+        <v>209</v>
       </c>
       <c r="R7" t="n">
-        <v>1911</v>
+        <v>1239</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1106,12 +1106,12 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1116991775</t>
+          <t>1266897442</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1116991775</t>
+          <t>https://m.place.naver.com/place/1266897442</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1121,20 +1121,36 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>바디쉬휘트니스 삼성중앙역점</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>bodyshe5@naver.com</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0507-1408-2010</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>주소</t>
+          <t>서울특별시 강남구 삼성로 571 케이빌딩 지하1층</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://blog.naver.com/bodyshe5/224041237261</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1144,12 +1160,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1165,17 +1181,17 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>599</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>355</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>954</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1184,12 +1200,12 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>6860803</t>
+          <t>1009390740</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/6860803</t>
+          <t>https://m.place.naver.com/place/1009390740</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1262,12 +1278,12 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>7065015</t>
+          <t>6860803</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7065015</t>
+          <t>https://m.place.naver.com/place/6860803</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1340,12 +1356,12 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>7423499</t>
+          <t>7065015</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7423499</t>
+          <t>https://m.place.naver.com/place/7065015</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1418,12 +1434,12 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>7161559</t>
+          <t>7423499</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7161559</t>
+          <t>https://m.place.naver.com/place/7423499</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1496,15 +1512,93 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
+          <t>7161559</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/7161559</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>주소</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
           <t>7476220</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>https://m.place.naver.com/place/7476220</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>2026-04-14</t>
         </is>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-25 00:00 | onda-hompage | 302 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강남_PT.xlsx
+++ b/naver-place-crawler/results_health/강남_PT.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -426,8 +426,8 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="7" max="7"/>
+    <col width="39" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
@@ -559,34 +559,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>헬스장</t>
+          <t>스포츠시설</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>헬스보이짐 필라걸 학동역점</t>
+          <t>청담짐 PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>healthboygym37@naver.com</t>
+          <t>cheongdamgym8@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1446-9059</t>
+          <t>0507-1332-0757</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 학동로 171 삼익악기빌딩 B1</t>
+          <t>서울특별시 강남구 도산대로81길 8 지하1층</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboygym37</t>
+          <t>https://blog.naver.com/cheongdamgym8</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -612,7 +612,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>2330</v>
+        <v>72</v>
       </c>
       <c r="Q2" t="n">
-        <v>1057</v>
+        <v>89</v>
       </c>
       <c r="R2" t="n">
-        <v>3387</v>
+        <v>161</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -636,17 +636,17 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1739218540</t>
+          <t>1729496529</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1739218540</t>
+          <t>https://m.place.naver.com/place/1729496529</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
@@ -658,29 +658,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>엑스퍼티짐 헬스 골프 역삼점</t>
+          <t>헬스보이짐&amp;필라걸&amp;골프인 선릉점</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>expurty@naver.com</t>
+          <t>healthboy42@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1338-8250</t>
+          <t>0507-1422-4228</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 테헤란로25길 7 창성재단빌딩 B1층 헬스 B2층 골프</t>
+          <t>서울특별시 강남구 테헤란로 317 동훈타워, B1층</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/expurty</t>
+          <t>https://www.instagram.com/healthboy42</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>574</v>
+        <v>686</v>
       </c>
       <c r="Q3" t="n">
-        <v>590</v>
+        <v>856</v>
       </c>
       <c r="R3" t="n">
-        <v>1164</v>
+        <v>1542</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,51 +730,51 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1327900562</t>
+          <t>1891416924</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1327900562</t>
+          <t>https://m.place.naver.com/place/1891416924</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>에이블짐 강남역점</t>
+          <t>헬스보이짐 필라걸 학동역점</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ablegym39@naver.com</t>
+          <t>healthboygym37@naver.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1352-2640</t>
+          <t>0507-1446-9059</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 강남대로 382 B2 에이블짐 강남역점</t>
+          <t>서울특별시 강남구 학동로 171 삼익악기빌딩 B1</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ablegym39</t>
+          <t>https://blog.naver.com/healthboygym37</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -809,13 +809,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>4576</v>
+        <v>2336</v>
       </c>
       <c r="Q4" t="n">
-        <v>3295</v>
+        <v>1138</v>
       </c>
       <c r="R4" t="n">
-        <v>7871</v>
+        <v>3474</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -824,17 +824,17 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1958479504</t>
+          <t>1739218540</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1958479504</t>
+          <t>https://m.place.naver.com/place/1739218540</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
@@ -846,29 +846,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>헬스보이짐 강남역점</t>
+          <t>에이블짐 압구정로데오점</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>healthboy352@naver.com</t>
+          <t>ablegym15@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0507-1443-0244</t>
+          <t>0507-1353-3036</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 테헤란로2길 27 패스트파이브빌딩 지하1층~지하2층</t>
+          <t>서울특별시 강남구 압구정로 320 극동Gallry B1 에이블짐</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboy352/224048963164</t>
+          <t>https://blog.naver.com/ablegym15</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -903,13 +903,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>1117</v>
+        <v>2612</v>
       </c>
       <c r="Q5" t="n">
-        <v>1517</v>
+        <v>1083</v>
       </c>
       <c r="R5" t="n">
-        <v>2634</v>
+        <v>3695</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -918,17 +918,17 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1650445992</t>
+          <t>1351701125</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1650445992</t>
+          <t>https://m.place.naver.com/place/1351701125</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
@@ -940,29 +940,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>밸류온피트니스 헬스&amp;PT 역삼점</t>
+          <t>에이블짐 강남역점</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pingpingwa@naver.com</t>
+          <t>ablegym39@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0507-1417-1245</t>
+          <t>0507-1352-2640</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 언주로 329 지하1층</t>
+          <t>서울특별시 강남구 강남대로 382 B2 에이블짐 강남역점</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/pingpingwa</t>
+          <t>https://blog.naver.com/ablegym39</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -997,13 +997,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>375</v>
+        <v>4599</v>
       </c>
       <c r="Q6" t="n">
-        <v>1527</v>
+        <v>3314</v>
       </c>
       <c r="R6" t="n">
-        <v>1902</v>
+        <v>7913</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1012,51 +1012,35 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1116991775</t>
+          <t>1958479504</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1116991775</t>
+          <t>https://m.place.naver.com/place/1958479504</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>헬스장</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>바디쉬휘트니스 언주역점</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>bodyshe_1@naver.com</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>0507-1417-1995</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 논현로 611 지하1층</t>
+          <t>주소</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/bodyshe_1</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1066,12 +1050,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1087,17 +1071,17 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>1030</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>209</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>1239</v>
+        <v>0</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1106,51 +1090,35 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1266897442</t>
+          <t>6860803</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1266897442</t>
+          <t>https://m.place.naver.com/place/6860803</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>헬스장</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>바디쉬휘트니스 삼성중앙역점</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>bodyshe5@naver.com</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0507-1408-2010</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 삼성로 571 케이빌딩 지하1층</t>
+          <t>주소</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/bodyshe5/224041237261</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1160,12 +1128,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1181,17 +1149,17 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>599</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>355</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>954</v>
+        <v>0</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1200,17 +1168,17 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1009390740</t>
+          <t>7065015</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1009390740</t>
+          <t>https://m.place.naver.com/place/7065015</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
@@ -1278,17 +1246,17 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>6860803</t>
+          <t>7423499</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/6860803</t>
+          <t>https://m.place.naver.com/place/7423499</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
@@ -1356,17 +1324,17 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>7065015</t>
+          <t>7161559</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7065015</t>
+          <t>https://m.place.naver.com/place/7161559</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
@@ -1434,173 +1402,17 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>7423499</t>
+          <t>7476220</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7423499</t>
+          <t>https://m.place.naver.com/place/7476220</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>주소</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>7161559</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>https://m.place.naver.com/place/7161559</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>주소</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>7476220</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>https://m.place.naver.com/place/7476220</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-26 04:00 | onda-hompage | 118 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강남_PT.xlsx
+++ b/naver-place-crawler/results_health/강남_PT.xlsx
@@ -421,13 +421,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="37" customWidth="1" min="7" max="7"/>
-    <col width="39" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
@@ -564,29 +564,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>청담짐 PT</t>
+          <t>탭핏 청담 피티 필라테스</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>cheongdamgym8@naver.com</t>
+          <t>tabhj@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1332-0757</t>
+          <t>0507-1425-8922</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 도산대로81길 8 지하1층</t>
+          <t>서울특별시 강남구 선릉로162길 41 지하1층</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/cheongdamgym8</t>
+          <t>https://open.kakao.com/o/sfTQ2cqe</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>72</v>
+        <v>217</v>
       </c>
       <c r="Q2" t="n">
-        <v>89</v>
+        <v>391</v>
       </c>
       <c r="R2" t="n">
-        <v>161</v>
+        <v>608</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -636,51 +636,51 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1729496529</t>
+          <t>1514885338</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1729496529</t>
+          <t>https://m.place.naver.com/place/1514885338</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>헬스장</t>
+          <t>스포츠시설</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>헬스보이짐&amp;필라걸&amp;골프인 선릉점</t>
+          <t>무브크래프트피티</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>healthboy42@naver.com</t>
+          <t>movecraft_pt@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1422-4228</t>
+          <t>0507-1355-9095</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 테헤란로 317 동훈타워, B1층</t>
+          <t>서울특별시 강남구 언주로113길 10 4층</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/healthboy42</t>
+          <t>https://blog.naver.com/movecraft_pt</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>686</v>
+        <v>16</v>
       </c>
       <c r="Q3" t="n">
-        <v>856</v>
+        <v>52</v>
       </c>
       <c r="R3" t="n">
-        <v>1542</v>
+        <v>68</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,56 +730,60 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1891416924</t>
+          <t>2064615220</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1891416924</t>
+          <t>https://m.place.naver.com/place/2064615220</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-26</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>헬스장</t>
+          <t>스포츠시설</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>헬스보이짐 필라걸 학동역점</t>
+          <t>버핏그라운드 PT 역삼GFC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>healthboygym37@naver.com</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>butfitground@naver.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>butfitseoul@butfitseoul.com</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1446-9059</t>
+          <t>0507-1310-0670</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 학동로 171 삼익악기빌딩 B1</t>
+          <t>서울 강남구 테헤란로 152 B1층</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboygym37</t>
+          <t>https://www.butfitground.com/4steppt</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -800,7 +804,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -809,13 +813,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>2336</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>1138</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>3474</v>
+        <v>0</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -824,17 +828,17 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1739218540</t>
+          <t>2080798868</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1739218540</t>
+          <t>https://m.place.naver.com/place/2080798868</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-26</t>
         </is>
       </c>
     </row>
@@ -846,29 +850,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>에이블짐 압구정로데오점</t>
+          <t>헬스보이짐 강남역점</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ablegym15@naver.com</t>
+          <t>healthboy352@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0507-1353-3036</t>
+          <t>0507-1443-0244</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 압구정로 320 극동Gallry B1 에이블짐</t>
+          <t>서울특별시 강남구 테헤란로2길 27 패스트파이브빌딩 지하1층~지하2층</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ablegym15</t>
+          <t>https://blog.naver.com/healthboy352/224048963164</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -903,13 +907,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>2612</v>
+        <v>1115</v>
       </c>
       <c r="Q5" t="n">
-        <v>1083</v>
+        <v>1527</v>
       </c>
       <c r="R5" t="n">
-        <v>3695</v>
+        <v>2642</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -918,17 +922,17 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1351701125</t>
+          <t>1650445992</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1351701125</t>
+          <t>https://m.place.naver.com/place/1650445992</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-26</t>
         </is>
       </c>
     </row>
@@ -940,29 +944,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>에이블짐 강남역점</t>
+          <t>에이블짐 압구정로데오점</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ablegym39@naver.com</t>
+          <t>ablegym15@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0507-1352-2640</t>
+          <t>0507-1353-3036</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 강남대로 382 B2 에이블짐 강남역점</t>
+          <t>서울특별시 강남구 압구정로 320 극동Gallry B1 에이블짐</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ablegym39</t>
+          <t>https://blog.naver.com/ablegym15</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -997,13 +1001,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>4599</v>
+        <v>2612</v>
       </c>
       <c r="Q6" t="n">
-        <v>3314</v>
+        <v>1085</v>
       </c>
       <c r="R6" t="n">
-        <v>7913</v>
+        <v>3697</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1012,17 +1016,17 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1958479504</t>
+          <t>1351701125</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1958479504</t>
+          <t>https://m.place.naver.com/place/1351701125</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-26</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1104,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-26</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1182,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-26</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1260,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-26</t>
         </is>
       </c>
     </row>
@@ -1324,17 +1328,17 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>7161559</t>
+          <t>7476220</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7161559</t>
+          <t>https://m.place.naver.com/place/7476220</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-26</t>
         </is>
       </c>
     </row>
@@ -1402,17 +1406,17 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>7476220</t>
+          <t>7161559</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7476220</t>
+          <t>https://m.place.naver.com/place/7161559</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-26 12:00 | onda-hompage | 122 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강남_PT.xlsx
+++ b/naver-place-crawler/results_health/강남_PT.xlsx
@@ -417,22 +417,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -564,34 +564,38 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>탭핏 청담 피티 필라테스</t>
+          <t>버핏그라운드 PT 도곡</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>tabhj@naver.com</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>butfitground@naver.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>butfitseoul@butfitseoul.com</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1425-8922</t>
+          <t>0507-1446-0895</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 선릉로162길 41 지하1층</t>
+          <t>서울 강남구 언주로30길 21 아카데미스위트빌딩 B2층</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://open.kakao.com/o/sfTQ2cqe</t>
+          <t>https://www.butfitground.com/4steppt</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -601,7 +605,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -621,13 +625,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>217</v>
+        <v>7</v>
       </c>
       <c r="Q2" t="n">
-        <v>391</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>608</v>
+        <v>7</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -636,12 +640,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1514885338</t>
+          <t>2007075506</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1514885338</t>
+          <t>https://m.place.naver.com/place/2007075506</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -653,34 +657,34 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>무브크래프트피티</t>
+          <t>헬스보이짐&amp;필라걸&amp;골프인 선릉점</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>movecraft_pt@naver.com</t>
+          <t>healthboy42@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1355-9095</t>
+          <t>0507-1422-4228</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 언주로113길 10 4층</t>
+          <t>서울 강남구 테헤란로 317 동훈타워, B1층</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/movecraft_pt</t>
+          <t>https://www.instagram.com/healthboy42</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -695,15 +699,19 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>https://talk.naver.com/ct/w4muek</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
           <t>X</t>
@@ -715,13 +723,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>16</v>
+        <v>686</v>
       </c>
       <c r="Q3" t="n">
-        <v>52</v>
+        <v>860</v>
       </c>
       <c r="R3" t="n">
-        <v>68</v>
+        <v>1546</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,12 +738,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2064615220</t>
+          <t>1891416924</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2064615220</t>
+          <t>https://m.place.naver.com/place/1891416924</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -752,38 +760,34 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>버핏그라운드 PT 역삼GFC</t>
+          <t>헬스보이짐 강남역점</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>butfitground@naver.com</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>butfitseoul@butfitseoul.com</t>
-        </is>
-      </c>
+          <t>healthboy352@naver.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1310-0670</t>
+          <t>0507-1443-0244</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>서울 강남구 테헤란로 152 B1층</t>
+          <t>서울 강남구 테헤란로2길 27 패스트파이브빌딩 지하1층~지하2층</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.butfitground.com/4steppt</t>
+          <t>https://blog.naver.com/healthboy352/224048963164</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -798,13 +802,17 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>https://talk.naver.com/ct/w4gs7y</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -813,13 +821,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>1115</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>1527</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>2642</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -828,12 +836,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2080798868</t>
+          <t>1650445992</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2080798868</t>
+          <t>https://m.place.naver.com/place/1650445992</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -850,29 +858,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>헬스보이짐 강남역점</t>
+          <t>에이블짐 압구정로데오점</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>healthboy352@naver.com</t>
+          <t>ablegym15@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0507-1443-0244</t>
+          <t>0507-1353-3036</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 테헤란로2길 27 패스트파이브빌딩 지하1층~지하2층</t>
+          <t>서울 강남구 압구정로 320 극동Gallry B1 에이블짐</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboy352/224048963164</t>
+          <t>https://blog.naver.com/ablegym15</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -892,10 +900,14 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://talk.naver.com/ct/w4ye97</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>X</t>
@@ -907,13 +919,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>1115</v>
+        <v>2612</v>
       </c>
       <c r="Q5" t="n">
-        <v>1527</v>
+        <v>1090</v>
       </c>
       <c r="R5" t="n">
-        <v>2642</v>
+        <v>3702</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -922,12 +934,12 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1650445992</t>
+          <t>1351701125</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1650445992</t>
+          <t>https://m.place.naver.com/place/1351701125</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -944,29 +956,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>에이블짐 압구정로데오점</t>
+          <t>에이블짐 강남역점</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ablegym15@naver.com</t>
+          <t>ablegym39@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0507-1353-3036</t>
+          <t>0507-1352-2640</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 압구정로 320 극동Gallry B1 에이블짐</t>
+          <t>서울 강남구 강남대로 382 B2 에이블짐 강남역점</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ablegym15</t>
+          <t>https://blog.naver.com/ablegym39</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -986,10 +998,14 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr"/>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>https://talk.naver.com/ct/w427p0</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr">
         <is>
           <t>X</t>
@@ -1001,13 +1017,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>2612</v>
+        <v>4601</v>
       </c>
       <c r="Q6" t="n">
-        <v>1085</v>
+        <v>3318</v>
       </c>
       <c r="R6" t="n">
-        <v>3697</v>
+        <v>7919</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1016,12 +1032,12 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1351701125</t>
+          <t>1958479504</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1351701125</t>
+          <t>https://m.place.naver.com/place/1958479504</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1031,20 +1047,36 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>헬스보이짐 필라걸 학동역점</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>healthboygym37@naver.com</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0507-1446-9059</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>주소</t>
+          <t>서울 강남구 학동로 171 삼익악기빌딩 B1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://blog.naver.com/healthboygym37</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1054,20 +1086,24 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr"/>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>https://talk.naver.com/ct/w4loja</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>X</t>
@@ -1075,17 +1111,17 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>2339</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>1161</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1094,12 +1130,12 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>6860803</t>
+          <t>1739218540</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/6860803</t>
+          <t>https://m.place.naver.com/place/1739218540</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1172,12 +1208,12 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>7065015</t>
+          <t>6860803</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7065015</t>
+          <t>https://m.place.naver.com/place/6860803</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1250,12 +1286,12 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>7423499</t>
+          <t>7065015</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7423499</t>
+          <t>https://m.place.naver.com/place/7065015</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1328,12 +1364,12 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>7476220</t>
+          <t>7423499</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7476220</t>
+          <t>https://m.place.naver.com/place/7423499</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1406,15 +1442,93 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
+          <t>7476220</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/7476220</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>주소</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
           <t>7161559</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>https://m.place.naver.com/place/7161559</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-26 20:00 | onda-hompage | 130 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강남_PT.xlsx
+++ b/naver-place-crawler/results_health/강남_PT.xlsx
@@ -417,22 +417,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="37" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -559,43 +559,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>버핏그라운드 PT 도곡</t>
+          <t>헬스보이짐 필라걸 학동역점</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>butfitground@naver.com</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>butfitseoul@butfitseoul.com</t>
-        </is>
-      </c>
+          <t>healthboygym37@naver.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1446-0895</t>
+          <t>0507-1446-9059</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>서울 강남구 언주로30길 21 아카데미스위트빌딩 B2층</t>
+          <t>서울특별시 강남구 학동로 171 삼익악기빌딩 B1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.butfitground.com/4steppt</t>
+          <t>https://blog.naver.com/healthboygym37</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -616,22 +612,22 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>O</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
       <c r="P2" t="n">
-        <v>7</v>
+        <v>2339</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>1161</v>
       </c>
       <c r="R2" t="n">
-        <v>7</v>
+        <v>3500</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -640,12 +636,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2007075506</t>
+          <t>1739218540</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2007075506</t>
+          <t>https://m.place.naver.com/place/1739218540</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -662,29 +658,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>헬스보이짐&amp;필라걸&amp;골프인 선릉점</t>
+          <t>바디쉬휘트니스 언주역점</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>healthboy42@naver.com</t>
+          <t>bodyshe_1@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1422-4228</t>
+          <t>0507-1417-1995</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>서울 강남구 테헤란로 317 동훈타워, B1층</t>
+          <t>서울특별시 강남구 논현로 611 지하1층</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/healthboy42</t>
+          <t>https://blog.naver.com/bodyshe_1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -699,37 +695,33 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>O</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4muek</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
       <c r="P3" t="n">
-        <v>686</v>
+        <v>1036</v>
       </c>
       <c r="Q3" t="n">
-        <v>860</v>
+        <v>276</v>
       </c>
       <c r="R3" t="n">
-        <v>1546</v>
+        <v>1312</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -738,12 +730,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1891416924</t>
+          <t>1266897442</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1891416924</t>
+          <t>https://m.place.naver.com/place/1266897442</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -760,29 +752,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>헬스보이짐 강남역점</t>
+          <t>에이블짐 압구정로데오점</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>healthboy352@naver.com</t>
+          <t>ablegym15@naver.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1443-0244</t>
+          <t>0507-1353-3036</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>서울 강남구 테헤란로2길 27 패스트파이브빌딩 지하1층~지하2층</t>
+          <t>서울특별시 강남구 압구정로 320 극동Gallry B1 에이블짐</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboy352/224048963164</t>
+          <t>https://blog.naver.com/ablegym15</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -802,32 +794,28 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
           <t>O</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4gs7y</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
       <c r="P4" t="n">
-        <v>1115</v>
+        <v>2612</v>
       </c>
       <c r="Q4" t="n">
-        <v>1527</v>
+        <v>1090</v>
       </c>
       <c r="R4" t="n">
-        <v>2642</v>
+        <v>3702</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -836,12 +824,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1650445992</t>
+          <t>1351701125</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1650445992</t>
+          <t>https://m.place.naver.com/place/1351701125</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -858,29 +846,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>에이블짐 압구정로데오점</t>
+          <t>에이블짐 강남역점</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ablegym15@naver.com</t>
+          <t>ablegym39@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0507-1353-3036</t>
+          <t>0507-1352-2640</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>서울 강남구 압구정로 320 극동Gallry B1 에이블짐</t>
+          <t>서울특별시 강남구 강남대로 382 B2 에이블짐 강남역점</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ablegym15</t>
+          <t>https://blog.naver.com/ablegym39</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -900,32 +888,28 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>O</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4ye97</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
       <c r="P5" t="n">
-        <v>2612</v>
+        <v>4601</v>
       </c>
       <c r="Q5" t="n">
-        <v>1090</v>
+        <v>3318</v>
       </c>
       <c r="R5" t="n">
-        <v>3702</v>
+        <v>7919</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -934,12 +918,12 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1351701125</t>
+          <t>1958479504</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1351701125</t>
+          <t>https://m.place.naver.com/place/1958479504</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -956,29 +940,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>에이블짐 강남역점</t>
+          <t>헬스보이짐 강남역점</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ablegym39@naver.com</t>
+          <t>healthboy352@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0507-1352-2640</t>
+          <t>0507-1443-0244</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>서울 강남구 강남대로 382 B2 에이블짐 강남역점</t>
+          <t>서울특별시 강남구 테헤란로2길 27 패스트파이브빌딩 지하1층~지하2층</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ablegym39</t>
+          <t>https://blog.naver.com/healthboy352/224048963164</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -998,32 +982,28 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>O</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w427p0</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
       <c r="P6" t="n">
-        <v>4601</v>
+        <v>1115</v>
       </c>
       <c r="Q6" t="n">
-        <v>3318</v>
+        <v>1527</v>
       </c>
       <c r="R6" t="n">
-        <v>7919</v>
+        <v>2642</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1032,12 +1012,12 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1958479504</t>
+          <t>1650445992</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1958479504</t>
+          <t>https://m.place.naver.com/place/1650445992</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1047,36 +1027,20 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>헬스장</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>헬스보이짐 필라걸 학동역점</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>healthboygym37@naver.com</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>0507-1446-9059</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>서울 강남구 학동로 171 삼익악기빌딩 B1</t>
+          <t>주소</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboygym37</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1086,24 +1050,20 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4loja</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>X</t>
@@ -1111,17 +1071,17 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>2339</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>1161</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1130,12 +1090,12 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1739218540</t>
+          <t>6860803</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1739218540</t>
+          <t>https://m.place.naver.com/place/6860803</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1208,12 +1168,12 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>6860803</t>
+          <t>7065015</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/6860803</t>
+          <t>https://m.place.naver.com/place/7065015</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1286,12 +1246,12 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>7065015</t>
+          <t>7423499</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7065015</t>
+          <t>https://m.place.naver.com/place/7423499</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1364,12 +1324,12 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>7423499</t>
+          <t>7476220</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7423499</t>
+          <t>https://m.place.naver.com/place/7476220</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1442,93 +1402,15 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>7476220</t>
+          <t>7161559</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7476220</t>
+          <t>https://m.place.naver.com/place/7161559</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
-        <is>
-          <t>2026-04-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>주소</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>7161559</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>https://m.place.naver.com/place/7161559</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-27 00:00 | onda-hompage | 117 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강남_PT.xlsx
+++ b/naver-place-crawler/results_health/강남_PT.xlsx
@@ -417,16 +417,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
@@ -624,10 +624,10 @@
         <v>2339</v>
       </c>
       <c r="Q2" t="n">
-        <v>1161</v>
+        <v>1169</v>
       </c>
       <c r="R2" t="n">
-        <v>3500</v>
+        <v>3508</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -658,29 +658,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>바디쉬휘트니스 언주역점</t>
+          <t>바디쉬휘트니스 삼성중앙역점</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>bodyshe_1@naver.com</t>
+          <t>bodyshe5@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1417-1995</t>
+          <t>0507-1408-2010</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 논현로 611 지하1층</t>
+          <t>서울특별시 강남구 삼성로 571 케이빌딩 지하1층</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/bodyshe_1</t>
+          <t>https://blog.naver.com/bodyshe5/224041237261</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>1036</v>
+        <v>608</v>
       </c>
       <c r="Q3" t="n">
-        <v>276</v>
+        <v>394</v>
       </c>
       <c r="R3" t="n">
-        <v>1312</v>
+        <v>1002</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,12 +730,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1266897442</t>
+          <t>1009390740</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1266897442</t>
+          <t>https://m.place.naver.com/place/1009390740</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -903,13 +903,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>4601</v>
+        <v>4603</v>
       </c>
       <c r="Q5" t="n">
-        <v>3318</v>
+        <v>3216</v>
       </c>
       <c r="R5" t="n">
-        <v>7919</v>
+        <v>7819</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1027,20 +1027,36 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>엑스퍼티짐 헬스 골프 역삼점</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>expurty@naver.com</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0507-1338-8250</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>주소</t>
+          <t>서울특별시 강남구 테헤란로25길 7 창성재단빌딩 B1층 헬스 B2층 골프</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://blog.naver.com/expurty</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1050,12 +1066,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1071,17 +1087,17 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>581</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>559</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>1140</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1090,12 +1106,12 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>6860803</t>
+          <t>1327900562</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/6860803</t>
+          <t>https://m.place.naver.com/place/1327900562</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1105,20 +1121,32 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>바디스짐 여성전용 강남구청점</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ooposohoo@naver.com</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>주소</t>
+          <t>서울특별시 강남구 선릉로146길 15 헤비히터빌딩 2층</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://blog.naver.com/ooposohoo</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1128,12 +1156,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1149,17 +1177,17 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>1299</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>405</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>1704</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1168,12 +1196,12 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>7065015</t>
+          <t>33938177</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7065015</t>
+          <t>https://m.place.naver.com/place/33938177</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1246,12 +1274,12 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>7423499</t>
+          <t>6860803</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7423499</t>
+          <t>https://m.place.naver.com/place/6860803</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1324,12 +1352,12 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>7476220</t>
+          <t>7065015</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7476220</t>
+          <t>https://m.place.naver.com/place/7065015</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1402,15 +1430,171 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
+          <t>7423499</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/7423499</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>주소</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>7476220</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/7476220</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>주소</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
           <t>7161559</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>https://m.place.naver.com/place/7161559</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-27 20:00 | onda-hompage | 140 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강남_PT.xlsx
+++ b/naver-place-crawler/results_health/강남_PT.xlsx
@@ -421,9 +421,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
@@ -432,7 +432,7 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -564,29 +564,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>헬스보이짐&amp;필라걸&amp;골프인 선릉점</t>
+          <t>바디스짐 여성전용 강남구청점</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>healthboy42@naver.com</t>
+          <t>ooposohoo@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>0507-1422-4228</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 테헤란로 317 동훈타워, B1층</t>
+          <t>서울특별시 강남구 선릉로146길 15 헤비히터빌딩 2층</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/healthboy42</t>
+          <t>https://blog.naver.com/ooposohoo</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -601,7 +597,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -621,13 +617,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>686</v>
+        <v>1299</v>
       </c>
       <c r="Q2" t="n">
-        <v>862</v>
+        <v>413</v>
       </c>
       <c r="R2" t="n">
-        <v>1548</v>
+        <v>1712</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -636,12 +632,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1891416924</t>
+          <t>33938177</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1891416924</t>
+          <t>https://m.place.naver.com/place/33938177</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -653,39 +649,43 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>헬스장</t>
+          <t>스포츠시설</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>헬스보이짐 필라걸 학동역점</t>
+          <t>버핏그라운드 PT 삼성</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>healthboygym37@naver.com</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>butfitground@naver.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>butfitseoul@butfitseoul.com</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1446-9059</t>
+          <t>0507-1304-1224</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 학동로 171 삼익악기빌딩 B1</t>
+          <t>서울특별시 강남구 삼성로 512 B2층</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboygym37</t>
+          <t>https://www.butfitground.com/4steppt</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -706,7 +706,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>2338</v>
+        <v>3</v>
       </c>
       <c r="Q3" t="n">
-        <v>1170</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>3508</v>
+        <v>3</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,12 +730,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1739218540</t>
+          <t>2058356975</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1739218540</t>
+          <t>https://m.place.naver.com/place/2058356975</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -752,34 +752,38 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>에이블짐 압구정로데오점</t>
+          <t>버핏그라운드 PT 논현</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ablegym15@naver.com</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>butfitground@naver.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>butfitseoul@butfitseoul.com</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1353-3036</t>
+          <t>0507-1406-5263</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 압구정로 320 극동Gallry B1 에이블짐</t>
+          <t>서울 강남구 언주로 641 펜트힐루 논현 지하1층</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ablegym15</t>
+          <t>https://www.butfitground.com/4steppt</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -794,13 +798,17 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>https://talk.naver.com/ct/w4d6fh</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -809,13 +817,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>2613</v>
+        <v>49</v>
       </c>
       <c r="Q4" t="n">
-        <v>1092</v>
+        <v>57</v>
       </c>
       <c r="R4" t="n">
-        <v>3705</v>
+        <v>106</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -824,12 +832,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1351701125</t>
+          <t>1826352348</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1351701125</t>
+          <t>https://m.place.naver.com/place/1826352348</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -846,29 +854,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>에이블짐 강남역점</t>
+          <t>에이블짐 압구정로데오점</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ablegym39@naver.com</t>
+          <t>ablegym15@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0507-1352-2640</t>
+          <t>0507-1353-3036</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 강남대로 382 B2 에이블짐 강남역점</t>
+          <t>서울특별시 강남구 압구정로 320 극동Gallry B1 에이블짐</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ablegym39</t>
+          <t>https://blog.naver.com/ablegym15</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -903,13 +911,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>4604</v>
+        <v>2613</v>
       </c>
       <c r="Q5" t="n">
-        <v>3218</v>
+        <v>1094</v>
       </c>
       <c r="R5" t="n">
-        <v>7822</v>
+        <v>3707</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -918,12 +926,12 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1958479504</t>
+          <t>1351701125</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1958479504</t>
+          <t>https://m.place.naver.com/place/1351701125</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -940,29 +948,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>헬스보이짐 강남역점</t>
+          <t>에이블짐 강남역점</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>healthboy352@naver.com</t>
+          <t>ablegym39@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0507-1443-0244</t>
+          <t>0507-1352-2640</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 테헤란로2길 27 패스트파이브빌딩 지하1층~지하2층</t>
+          <t>서울특별시 강남구 강남대로 382 B2 에이블짐 강남역점</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboy352/224048963164</t>
+          <t>https://blog.naver.com/ablegym39</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -997,13 +1005,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>1115</v>
+        <v>4604</v>
       </c>
       <c r="Q6" t="n">
-        <v>1527</v>
+        <v>3218</v>
       </c>
       <c r="R6" t="n">
-        <v>2642</v>
+        <v>7822</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1012,12 +1020,12 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1650445992</t>
+          <t>1958479504</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1650445992</t>
+          <t>https://m.place.naver.com/place/1958479504</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1029,34 +1037,34 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>헬스장</t>
+          <t>스포츠시설</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>바디쉬휘트니스 언주역점</t>
+          <t>헬스보이짐 강남역점</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>bodyshe_1@naver.com</t>
+          <t>healthboy352@naver.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0507-1417-1995</t>
+          <t>0507-1443-0244</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 논현로 611 지하1층</t>
+          <t>서울특별시 강남구 테헤란로2길 27 패스트파이브빌딩 지하1층~지하2층</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/bodyshe_1</t>
+          <t>https://blog.naver.com/healthboy352/224048963164</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1091,13 +1099,13 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>1036</v>
+        <v>1115</v>
       </c>
       <c r="Q7" t="n">
-        <v>283</v>
+        <v>1528</v>
       </c>
       <c r="R7" t="n">
-        <v>1319</v>
+        <v>2643</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1106,12 +1114,12 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1266897442</t>
+          <t>1650445992</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1266897442</t>
+          <t>https://m.place.naver.com/place/1650445992</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1128,29 +1136,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>바디쉬휘트니스 삼성중앙역점</t>
+          <t>헬스보이짐 필라걸 학동역점</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>bodyshe5@naver.com</t>
+          <t>healthboygym37@naver.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0507-1408-2010</t>
+          <t>0507-1446-9059</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 삼성로 571 케이빌딩 지하1층</t>
+          <t>서울특별시 강남구 학동로 171 삼익악기빌딩 B1</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/bodyshe5/224041237261</t>
+          <t>https://blog.naver.com/healthboygym37</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1185,13 +1193,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>608</v>
+        <v>2338</v>
       </c>
       <c r="Q8" t="n">
-        <v>394</v>
+        <v>1170</v>
       </c>
       <c r="R8" t="n">
-        <v>1002</v>
+        <v>3508</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1200,12 +1208,12 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1009390740</t>
+          <t>1739218540</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1009390740</t>
+          <t>https://m.place.naver.com/place/1739218540</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-28 04:00 | onda-hompage | 136 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강남_PT.xlsx
+++ b/naver-place-crawler/results_health/강남_PT.xlsx
@@ -422,8 +422,8 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
@@ -432,7 +432,7 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -559,30 +559,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>헬스장</t>
+          <t>스포츠시설</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>바디스짐 여성전용 강남구청점</t>
+          <t>탭핏 청담 피티 필라테스</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ooposohoo@naver.com</t>
+          <t>tabhj@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0507-1425-8922</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 선릉로146길 15 헤비히터빌딩 2층</t>
+          <t>서울특별시 강남구 선릉로162길 41 지하1층</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ooposohoo</t>
+          <t>https://open.kakao.com/o/sfTQ2cqe</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -597,7 +601,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -608,7 +612,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -617,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>1299</v>
+        <v>217</v>
       </c>
       <c r="Q2" t="n">
-        <v>413</v>
+        <v>400</v>
       </c>
       <c r="R2" t="n">
-        <v>1712</v>
+        <v>617</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -632,60 +636,56 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>33938177</t>
+          <t>1514885338</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/33938177</t>
+          <t>https://m.place.naver.com/place/1514885338</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>버핏그라운드 PT 삼성</t>
+          <t>바디쉬휘트니스 삼성중앙역점</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>butfitground@naver.com</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>butfitseoul@butfitseoul.com</t>
-        </is>
-      </c>
+          <t>bodyshe5@naver.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1304-1224</t>
+          <t>0507-1408-2010</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 삼성로 512 B2층</t>
+          <t>서울특별시 강남구 삼성로 571 케이빌딩 지하1층</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.butfitground.com/4steppt</t>
+          <t>https://blog.naver.com/bodyshe5/224041237261</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -706,7 +706,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>3</v>
+        <v>609</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>394</v>
       </c>
       <c r="R3" t="n">
-        <v>3</v>
+        <v>1003</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,60 +730,52 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2058356975</t>
+          <t>1009390740</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2058356975</t>
+          <t>https://m.place.naver.com/place/1009390740</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>버핏그라운드 PT 논현</t>
+          <t>바디스짐 여성전용 강남구청점</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>butfitground@naver.com</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>butfitseoul@butfitseoul.com</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>0507-1406-5263</t>
-        </is>
-      </c>
+          <t>ooposohoo@naver.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>서울 강남구 언주로 641 펜트힐루 논현 지하1층</t>
+          <t>서울특별시 강남구 선릉로146길 15 헤비히터빌딩 2층</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.butfitground.com/4steppt</t>
+          <t>https://blog.naver.com/ooposohoo</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -798,17 +790,13 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4d6fh</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -817,13 +805,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>49</v>
+        <v>1299</v>
       </c>
       <c r="Q4" t="n">
-        <v>57</v>
+        <v>413</v>
       </c>
       <c r="R4" t="n">
-        <v>106</v>
+        <v>1712</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -832,17 +820,17 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1826352348</t>
+          <t>33938177</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1826352348</t>
+          <t>https://m.place.naver.com/place/33938177</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -911,13 +899,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>2613</v>
+        <v>2614</v>
       </c>
       <c r="Q5" t="n">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="R5" t="n">
-        <v>3707</v>
+        <v>3709</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -936,7 +924,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1018,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1112,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1136,29 +1124,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>헬스보이짐 필라걸 학동역점</t>
+          <t>바디쉬휘트니스 학동역점</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>healthboygym37@naver.com</t>
+          <t>bodyshe3@naver.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0507-1446-9059</t>
+          <t>0507-1378-2066</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 학동로 171 삼익악기빌딩 B1</t>
+          <t>서울특별시 강남구 학동로28길 5 지하1층</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboygym37</t>
+          <t>https://blog.naver.com/bodyshe3</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1193,13 +1181,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>2338</v>
+        <v>1186</v>
       </c>
       <c r="Q8" t="n">
-        <v>1170</v>
+        <v>602</v>
       </c>
       <c r="R8" t="n">
-        <v>3508</v>
+        <v>1788</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1208,17 +1196,17 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1739218540</t>
+          <t>1188704844</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1739218540</t>
+          <t>https://m.place.naver.com/place/1188704844</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1284,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1362,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1440,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1518,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1596,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-29 00:00 | onda-hompage | 111 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강남_PT.xlsx
+++ b/naver-place-crawler/results_health/강남_PT.xlsx
@@ -417,12 +417,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -559,34 +559,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>탭핏 청담 피티 필라테스</t>
+          <t>인어스휘트니스 헬스 PT &amp; 필라테스 골프 삼성점</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>tabhj@naver.com</t>
+          <t>inus_fitness01@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1425-8922</t>
+          <t>0507-1418-2225</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 선릉로162길 41 지하1층</t>
+          <t>서울특별시 강남구 영동대로 602 미켈란107빌딩 지하2층</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://open.kakao.com/o/sfTQ2cqe</t>
+          <t>https://blog.naver.com/inus_fitness01</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -612,7 +612,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>217</v>
+        <v>681</v>
       </c>
       <c r="Q2" t="n">
-        <v>400</v>
+        <v>962</v>
       </c>
       <c r="R2" t="n">
-        <v>617</v>
+        <v>1643</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -636,12 +636,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1514885338</t>
+          <t>35532894</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1514885338</t>
+          <t>https://m.place.naver.com/place/35532894</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -658,29 +658,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>바디쉬휘트니스 삼성중앙역점</t>
+          <t>헬스보이짐 필라걸 학동역점</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>bodyshe5@naver.com</t>
+          <t>healthboygym37@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1408-2010</t>
+          <t>0507-1446-9059</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 삼성로 571 케이빌딩 지하1층</t>
+          <t>서울특별시 강남구 학동로 171 삼익악기빌딩 B1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/bodyshe5/224041237261</t>
+          <t>https://blog.naver.com/healthboygym37</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>609</v>
+        <v>2338</v>
       </c>
       <c r="Q3" t="n">
-        <v>394</v>
+        <v>1171</v>
       </c>
       <c r="R3" t="n">
-        <v>1003</v>
+        <v>3509</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,12 +730,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1009390740</t>
+          <t>1739218540</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1009390740</t>
+          <t>https://m.place.naver.com/place/1739218540</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -752,25 +752,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>바디스짐 여성전용 강남구청점</t>
+          <t>바디쉬휘트니스 언주역점</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ooposohoo@naver.com</t>
+          <t>bodyshe_1@naver.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0507-1417-1995</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 선릉로146길 15 헤비히터빌딩 2층</t>
+          <t>서울특별시 강남구 논현로 611 지하1층</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ooposohoo</t>
+          <t>https://blog.naver.com/bodyshe_1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -805,13 +809,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>1299</v>
+        <v>1037</v>
       </c>
       <c r="Q4" t="n">
-        <v>413</v>
+        <v>282</v>
       </c>
       <c r="R4" t="n">
-        <v>1712</v>
+        <v>1319</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -820,12 +824,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>33938177</t>
+          <t>1266897442</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/33938177</t>
+          <t>https://m.place.naver.com/place/1266897442</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -899,13 +903,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>2614</v>
+        <v>2615</v>
       </c>
       <c r="Q5" t="n">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="R5" t="n">
-        <v>3709</v>
+        <v>3711</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -996,10 +1000,10 @@
         <v>4604</v>
       </c>
       <c r="Q6" t="n">
-        <v>3218</v>
+        <v>3219</v>
       </c>
       <c r="R6" t="n">
-        <v>7822</v>
+        <v>7823</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1090,10 +1094,10 @@
         <v>1115</v>
       </c>
       <c r="Q7" t="n">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="R7" t="n">
-        <v>2643</v>
+        <v>2644</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1117,36 +1121,20 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>헬스장</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>바디쉬휘트니스 학동역점</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>bodyshe3@naver.com</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0507-1378-2066</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 학동로28길 5 지하1층</t>
+          <t>주소</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/bodyshe3</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1156,12 +1144,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1177,17 +1165,17 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>1186</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>602</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>1788</v>
+        <v>0</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1196,12 +1184,12 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1188704844</t>
+          <t>6860803</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1188704844</t>
+          <t>https://m.place.naver.com/place/6860803</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1274,12 +1262,12 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>6860803</t>
+          <t>7065015</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/6860803</t>
+          <t>https://m.place.naver.com/place/7065015</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1352,12 +1340,12 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>7065015</t>
+          <t>7423499</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7065015</t>
+          <t>https://m.place.naver.com/place/7423499</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1430,12 +1418,12 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>7423499</t>
+          <t>7476220</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7423499</t>
+          <t>https://m.place.naver.com/place/7476220</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1508,93 +1496,15 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>7476220</t>
+          <t>7161559</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7476220</t>
+          <t>https://m.place.naver.com/place/7161559</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>주소</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>7161559</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>https://m.place.naver.com/place/7161559</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-29 04:00 | onda-hompage | 137 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강남_PT.xlsx
+++ b/naver-place-crawler/results_health/강남_PT.xlsx
@@ -417,13 +417,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:V14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
@@ -559,34 +559,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>헬스장</t>
+          <t>스포츠시설</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>인어스휘트니스 헬스 PT &amp; 필라테스 골프 삼성점</t>
+          <t>청담짐 PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>inus_fitness01@naver.com</t>
+          <t>cheongdamgym8@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1418-2225</t>
+          <t>0507-1332-0757</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 영동대로 602 미켈란107빌딩 지하2층</t>
+          <t>서울특별시 강남구 도산대로81길 8 지하1층</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/inus_fitness01</t>
+          <t>https://blog.naver.com/cheongdamgym8</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -612,7 +612,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>681</v>
+        <v>73</v>
       </c>
       <c r="Q2" t="n">
-        <v>962</v>
+        <v>89</v>
       </c>
       <c r="R2" t="n">
-        <v>1643</v>
+        <v>162</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -636,56 +636,60 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>35532894</t>
+          <t>1729496529</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/35532894</t>
+          <t>https://m.place.naver.com/place/1729496529</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>헬스장</t>
+          <t>스포츠시설</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>헬스보이짐 필라걸 학동역점</t>
+          <t>버핏그라운드 PT 삼성</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>healthboygym37@naver.com</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>butfitground@naver.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>butfitseoul@butfitseoul.com</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1446-9059</t>
+          <t>0507-1304-1224</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 학동로 171 삼익악기빌딩 B1</t>
+          <t>서울특별시 강남구 삼성로 512 B2층</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboygym37</t>
+          <t>https://www.butfitground.com/4steppt</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -706,7 +710,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -715,13 +719,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>2338</v>
+        <v>3</v>
       </c>
       <c r="Q3" t="n">
-        <v>1171</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>3509</v>
+        <v>3</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,56 +734,60 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1739218540</t>
+          <t>2058356975</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1739218540</t>
+          <t>https://m.place.naver.com/place/2058356975</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>헬스장</t>
+          <t>스포츠시설</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>바디쉬휘트니스 언주역점</t>
+          <t>버핏그라운드 PT 도곡</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>bodyshe_1@naver.com</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>butfitground@naver.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>butfitseoul@butfitseoul.com</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1417-1995</t>
+          <t>0507-1446-0895</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 논현로 611 지하1층</t>
+          <t>서울특별시 강남구 언주로30길 21 아카데미스위트빌딩 B2층</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/bodyshe_1</t>
+          <t>https://www.butfitground.com/4steppt</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -800,7 +808,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -809,13 +817,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>1037</v>
+        <v>7</v>
       </c>
       <c r="Q4" t="n">
-        <v>282</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>1319</v>
+        <v>7</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -824,17 +832,17 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1266897442</t>
+          <t>2007075506</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1266897442</t>
+          <t>https://m.place.naver.com/place/2007075506</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -928,7 +936,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -1000,10 +1008,10 @@
         <v>4604</v>
       </c>
       <c r="Q6" t="n">
-        <v>3219</v>
+        <v>3220</v>
       </c>
       <c r="R6" t="n">
-        <v>7823</v>
+        <v>7824</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1022,7 +1030,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -1116,25 +1124,45 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>버핏그라운드 도곡</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>butfitground@naver.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>butfitseoul@butfitseoul.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0507-1365-3624</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>주소</t>
+          <t>서울특별시 강남구 언주로30길 21 아카데미스위트빌딩 B2층</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://pt.butfitground.com/</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1144,12 +1172,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1160,22 +1188,22 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>1966</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>385</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>2351</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1184,35 +1212,51 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>6860803</t>
+          <t>1342122485</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/6860803</t>
+          <t>https://m.place.naver.com/place/1342122485</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>바디쉬휘트니스 삼성중앙역점</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>bodyshe5@naver.com</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0507-1408-2010</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>주소</t>
+          <t>서울특별시 강남구 삼성로 571 케이빌딩 지하1층</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://blog.naver.com/bodyshe5/224041237261</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1222,12 +1266,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1243,17 +1287,17 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>616</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>394</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>1010</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1262,17 +1306,17 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>7065015</t>
+          <t>1009390740</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7065015</t>
+          <t>https://m.place.naver.com/place/1009390740</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -1340,17 +1384,17 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>7423499</t>
+          <t>6860803</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7423499</t>
+          <t>https://m.place.naver.com/place/6860803</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -1418,17 +1462,17 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>7476220</t>
+          <t>7065015</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7476220</t>
+          <t>https://m.place.naver.com/place/7065015</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -1496,17 +1540,173 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
+          <t>7423499</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/7423499</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>주소</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>7476220</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/7476220</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>주소</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
           <t>7161559</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>https://m.place.naver.com/place/7161559</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-29 12:00 | onda-hompage | 117 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강남_PT.xlsx
+++ b/naver-place-crawler/results_health/강남_PT.xlsx
@@ -417,12 +417,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V14"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -559,34 +559,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>청담짐 PT</t>
+          <t>인어스휘트니스 헬스 PT &amp; 필라테스 골프 삼성점</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>cheongdamgym8@naver.com</t>
+          <t>inus_fitness01@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1332-0757</t>
+          <t>0507-1418-2225</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 도산대로81길 8 지하1층</t>
+          <t>서울특별시 강남구 영동대로 602 미켈란107빌딩 지하2층</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/cheongdamgym8</t>
+          <t>https://blog.naver.com/inus_fitness01</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -612,7 +612,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>73</v>
+        <v>681</v>
       </c>
       <c r="Q2" t="n">
-        <v>89</v>
+        <v>962</v>
       </c>
       <c r="R2" t="n">
-        <v>162</v>
+        <v>1643</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -636,12 +636,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1729496529</t>
+          <t>35532894</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1729496529</t>
+          <t>https://m.place.naver.com/place/35532894</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -751,43 +751,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>버핏그라운드 PT 도곡</t>
+          <t>헬스보이짐&amp;필라걸&amp;골프인 선릉점</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>butfitground@naver.com</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>butfitseoul@butfitseoul.com</t>
-        </is>
-      </c>
+          <t>healthboy42@naver.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1446-0895</t>
+          <t>0507-1422-4228</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 언주로30길 21 아카데미스위트빌딩 B2층</t>
+          <t>서울특별시 강남구 테헤란로 317 동훈타워, B1층</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.butfitground.com/4steppt</t>
+          <t>https://www.instagram.com/healthboy42</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -797,7 +793,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -808,7 +804,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -817,13 +813,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>7</v>
+        <v>686</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>867</v>
       </c>
       <c r="R4" t="n">
-        <v>7</v>
+        <v>1553</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -832,12 +828,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2007075506</t>
+          <t>1891416924</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2007075506</t>
+          <t>https://m.place.naver.com/place/1891416924</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -914,10 +910,10 @@
         <v>2615</v>
       </c>
       <c r="Q5" t="n">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="R5" t="n">
-        <v>3711</v>
+        <v>3712</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1129,40 +1125,20 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>헬스장</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>버핏그라운드 도곡</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>butfitground@naver.com</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>butfitseoul@butfitseoul.com</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0507-1365-3624</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 언주로30길 21 아카데미스위트빌딩 B2층</t>
+          <t>주소</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://pt.butfitground.com/</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1172,12 +1148,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1188,22 +1164,22 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>1966</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>385</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>2351</v>
+        <v>0</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1212,12 +1188,12 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1342122485</t>
+          <t>6860803</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1342122485</t>
+          <t>https://m.place.naver.com/place/6860803</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1227,36 +1203,20 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>헬스장</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>바디쉬휘트니스 삼성중앙역점</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>bodyshe5@naver.com</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>0507-1408-2010</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 삼성로 571 케이빌딩 지하1층</t>
+          <t>주소</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/bodyshe5/224041237261</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1266,12 +1226,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1287,17 +1247,17 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>616</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>394</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>1010</v>
+        <v>0</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1306,12 +1266,12 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1009390740</t>
+          <t>7065015</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1009390740</t>
+          <t>https://m.place.naver.com/place/7065015</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1384,12 +1344,12 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>6860803</t>
+          <t>7423499</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/6860803</t>
+          <t>https://m.place.naver.com/place/7423499</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1462,12 +1422,12 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>7065015</t>
+          <t>7476220</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7065015</t>
+          <t>https://m.place.naver.com/place/7476220</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1540,171 +1500,15 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>7423499</t>
+          <t>7161559</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/7423499</t>
+          <t>https://m.place.naver.com/place/7161559</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
-        <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>주소</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>7476220</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>https://m.place.naver.com/place/7476220</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>주소</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>7161559</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>https://m.place.naver.com/place/7161559</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>

</xml_diff>